<commit_message>
Revise manuscript to reflect systematic mapping study methodology and findings
- Updated the title and abstract to clarify the study as a systematic mapping study rather than a literature review.
- Enhanced the introduction to position the study against existing literature and articulate the unique contributions of the research.
- Revised methodology to include detailed descriptions of the LLM-assisted screening process and human validation results, including kappa statistics and Lost Evidence metrics.
- Adjusted findings to reflect the confirmed primary studies and their implications for future research, particularly regarding the PATHCAST framework.
- Added new references and updated eligibility criteria for the literature search, ensuring alignment with the revised study scope.
</commit_message>
<xml_diff>
--- a/results/human_validation/ft_pdf_links_needed.xlsx
+++ b/results/human_validation/ft_pdf_links_needed.xlsx
@@ -493,7 +493,6 @@
           <t>IEEE International Conference on Program Comprehension</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>url</t>
@@ -524,7 +523,6 @@
           <t>Information Systems</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -555,7 +553,6 @@
           <t>Communications in Computer and Information Science</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>doi</t>
@@ -586,7 +583,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>doi</t>
@@ -617,7 +613,6 @@
           <t>Advances in Intelligent and Soft Computing</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>doi</t>
@@ -648,7 +643,6 @@
           <t>Proceedings 12th Pacific Rim International Symposium on Dependable Computing Prdc 2006</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>doi</t>
@@ -679,7 +673,6 @@
           <t>Enase 2014 Proceedings of the 9th International Conference on Evaluation of Novel Approaches to Software Engineering</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -710,7 +703,6 @@
           <t>Proceedings 2020 IEEE 24th International Enterprise Distributed Object Computing Conference Edoc 2020</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>url</t>
@@ -741,7 +733,6 @@
           <t>Proceedings International Computer Software and Applications Conference</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>doi</t>
@@ -772,7 +763,6 @@
           <t>International Journal of Reliability Quality and Safety Engineering</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>doi</t>
@@ -803,7 +793,11 @@
           <t>International Journal of Software Engineering and Knowledge Engineering</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>doi</t>
@@ -834,7 +828,6 @@
           <t>2012 IEEE 5th International Conference on Advanced Computational Intelligence Icaci 2012</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>doi</t>
@@ -865,7 +858,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>doi</t>
@@ -896,7 +888,6 @@
           <t>Companion Proceedings of the 36th International Conference on Software Engineering (ICSE Companion 2014)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>doi</t>
@@ -927,7 +918,6 @@
           <t>Proceedings of the Iadis International Conference Information Systems 2012 is 2012</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>url</t>
@@ -958,7 +948,6 @@
           <t>Advances and Innovations in Systems Computing Sciences and Software Engineering</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>doi</t>
@@ -991,7 +980,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>no-ok</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1024,7 +1013,6 @@
           <t>ACM International Conference Proceeding Series</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -1055,7 +1043,6 @@
           <t>Tsinghua Science and Technology</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -1086,7 +1073,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1117,7 +1103,6 @@
           <t>Icic Express Letters Part B Applications</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1148,7 +1133,6 @@
           <t>Simulation Modelling Practice and Theory</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1179,7 +1163,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>url</t>
@@ -1210,7 +1193,6 @@
           <t>Proceedings of the IEEE International Conference on Software Engineering and Service Sciences Icsess</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1241,7 +1223,6 @@
           <t>Statistics</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1272,7 +1253,6 @@
           <t>Springerbriefs in Applied Sciences and Technology</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1305,7 +1285,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>no-ok</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1338,7 +1318,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1369,7 +1348,6 @@
           <t>Ase 2017 Proceedings of the 32nd IEEE ACM International Conference on Automated Software Engineering</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1400,7 +1378,6 @@
           <t>Proceedings 2021 IEEE ACM 18th International Conference on Mining Software Repositories MSR 2021</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>url</t>
@@ -1431,7 +1408,6 @@
           <t>Proceedings 2025 9th International Conference on Management Engineering Software Engineering and Service Sciences Icmss 2025</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>url</t>
@@ -1462,7 +1438,11 @@
           <t>Advances in Intelligent Systems and Computing</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>no-access</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1493,7 +1473,6 @@
           <t>25th European Modeling and Simulation Symposium Emss 2013</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>url</t>
@@ -1524,7 +1503,6 @@
           <t>Icqr 2007 Proceedings of the 5th International Conference on Quality and Reliability</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>url</t>
@@ -1555,7 +1533,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>url</t>
@@ -1586,7 +1563,6 @@
           <t>Proceedings of the 2014 International Conference on Software and System Process</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1617,7 +1593,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1648,7 +1623,6 @@
           <t>Proceedings of the 38th International Conference on Software Engineering Companion (ICSE '16)</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1679,7 +1653,11 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1710,7 +1688,6 @@
           <t>International Journal of System Assurance Engineering and Management</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1743,7 +1720,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>no-ok</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1776,7 +1753,6 @@
           <t>Communications in Computer and Information Science</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -1807,7 +1783,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>url</t>
@@ -1838,7 +1813,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1869,7 +1843,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>url</t>
@@ -1900,7 +1873,6 @@
           <t>Computational Statistics and Data Analysis</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1931,7 +1903,11 @@
           <t>Seke 2011 Proceedings of the 23rd International Conference on Software Engineering and Knowledge Engineering</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>url</t>
@@ -1962,7 +1938,6 @@
           <t>36th International Conference on Software Engineering ICSE Companion 2014 Proceedings</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>doi</t>
@@ -1993,7 +1968,6 @@
           <t>Smart Innovation Systems and Technologies</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2024,7 +1998,11 @@
           <t>Procedia Computer Science</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>no-ok</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -2055,7 +2033,11 @@
           <t>ACM Transactions on Software Engineering and Methodology (TOSEM)</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -2086,7 +2068,6 @@
           <t>International Journal of System Assurance Engineering and Management</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2117,7 +2098,6 @@
           <t>Proceedings International Symposium on Parallel Architectures Algorithms and Programming Paap</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2148,7 +2128,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>url</t>
@@ -2179,7 +2158,6 @@
           <t>Proceedings International Computer Software and Applications Conference</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2210,7 +2188,6 @@
           <t>Simulation Series</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>url</t>
@@ -2241,7 +2218,6 @@
           <t>Proceedings International Conference on Software Engineering</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2272,7 +2248,6 @@
           <t>Advances in Intelligent and Soft Computing</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2303,7 +2278,6 @@
           <t>Proceedings of the 2015 IEEE 19th International Conference on Computer Supported Cooperative Work in Design Cscwd 2015</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2334,7 +2308,6 @@
           <t>Epic Series in Computing</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2365,7 +2338,6 @@
           <t>Proceedings Winter Simulation Conference</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -2396,7 +2368,6 @@
           <t>Proceedings 2019 International Conference on Process Mining Icpm 2019</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>url</t>
@@ -2427,7 +2398,6 @@
           <t>Proceedings 2022 4th International Conference on Process Mining Icpm 2022</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>url</t>
@@ -2458,7 +2428,11 @@
           <t>Proceedings 2016 12th International ACM SIGSOFT Conference on Quality of Software Architectures Qosa 2016</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2489,13 +2463,11 @@
           <t>Proceedings of the International Conference on Software and System Process</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2516,7 +2488,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -2547,7 +2518,6 @@
           <t>Wiley Interdisciplinary Reviews Computational Statistics</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2578,7 +2548,6 @@
           <t>International Journal of Performability Engineering</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -2609,7 +2578,6 @@
           <t>Bmsd 2017 Proceedings of the 7th International Symposium on Business Modeling and Software Design</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -2640,7 +2608,6 @@
           <t>Proceedings 2025 IEEE ACM 22nd International Conference on Mining Software Repositories MSR 2025</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -2671,7 +2638,6 @@
           <t>Computer Systems and Software Engineering Concepts Methodologies Tools and Applications</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2702,7 +2668,11 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>url</t>
@@ -2733,7 +2703,6 @@
           <t>Proceedings 5th International Conference on Software Engineering Advances Icsea 2010</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2764,7 +2733,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2795,7 +2763,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>url</t>
@@ -2826,7 +2793,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>url</t>
@@ -2857,7 +2823,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -2888,7 +2853,6 @@
           <t>Proceedings International Conference on Software Engineering</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2919,7 +2883,6 @@
           <t>International Journal of Computational Science and Engineering</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>doi</t>
@@ -2950,7 +2913,6 @@
           <t>Proceedings International Conference on Software Engineering</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>url</t>
@@ -2981,7 +2943,6 @@
           <t>Information and Software Technology</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -3012,7 +2973,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>url</t>
@@ -3043,7 +3003,6 @@
           <t>Proceedings IEEE International Enterprise Distributed Object Computing Workshop Edoc</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>url</t>
@@ -3074,7 +3033,6 @@
           <t>Communications in Computer and Information Science</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3105,7 +3063,6 @@
           <t>Proceedings 15th Euromicro Conference on Digital System Design Dsd 2012</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3136,7 +3093,11 @@
           <t>2016 International Conference on High Performance Computing and Simulation Hpcs 2016</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3167,7 +3128,6 @@
           <t>Proceedings International Conference on Software Engineering</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -3198,7 +3158,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>url</t>
@@ -3229,7 +3188,11 @@
           <t>Proceedings 2022 4th International Conference on Process Mining Icpm 2022</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -3260,7 +3223,6 @@
           <t>Applied Intelligence</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3291,7 +3253,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>url</t>
@@ -3322,7 +3283,6 @@
           <t>Information and Software Technology</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3353,7 +3313,11 @@
           <t>Proceedings 2010 IEEE International Conference on Software Engineering and Service Sciences Icsess 2010</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3384,7 +3348,6 @@
           <t>Iet Software</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3415,7 +3378,6 @@
           <t>Lecture Notes in Engineering and Computer Science</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>url</t>
@@ -3446,7 +3408,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>url</t>
@@ -3477,7 +3438,6 @@
           <t>Proceedings of the American Control Conference</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>url</t>
@@ -3508,7 +3468,6 @@
           <t>International Journal of Computer Applications in Technology</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3539,7 +3498,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -3570,7 +3528,6 @@
           <t>2009 International Conference on Research Challenges in Computer Science</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3601,7 +3558,11 @@
           <t>Proceedings 2010 2nd Wri World Congress on Software Engineering Wcse 2010</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F102" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3632,7 +3593,6 @@
           <t>IEEE Transactions on Software Engineering</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3663,7 +3623,6 @@
           <t>Proceedings of the 2014 International Conference on Software and System Process</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3694,7 +3653,6 @@
           <t>IEEE International Working Conference on Mining Software Repositories</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3725,7 +3683,6 @@
           <t>Proceedings of the 1st International Technology Management Conference Itmc 2011</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3756,7 +3713,6 @@
           <t>Lecture Notes in Computer Science Including Subseries Lecture Notes in Artificial Intelligence and Lecture Notes in Bioinformatics</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3787,7 +3743,6 @@
           <t>Companion Proceedings of the 36th International Conference on Software Engineering (ICSE Companion 2014)</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3818,7 +3773,6 @@
           <t>Software Testing Verification and Reliability</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>doi</t>
@@ -3849,7 +3803,6 @@
           <t>International Journal of Performability Engineering</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -3880,7 +3833,6 @@
           <t>Proceedings International Computer Software and Applications Conference</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>url</t>
@@ -3911,7 +3863,6 @@
           <t>39th International Annual Conference of the American Society for Engineering Management Asem 2018 Bridging the Gap Between Engineering and Business</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>url</t>
@@ -3942,7 +3893,6 @@
           <t>Inforsid 2016 Actes Du 8e Forum Jeunes Chercheurs Du Congres Inforsid</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>url</t>
@@ -4008,7 +3958,6 @@
           <t>Information Systems</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4039,7 +3988,6 @@
           <t>Proceedings 2024 6th International Conference on Process Mining Icpm 2024</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>url</t>
@@ -4070,7 +4018,6 @@
           <t>2009 International Conference on Machine Learning and Applications</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4101,7 +4048,6 @@
           <t>Proceedings International Symposium on Software Reliability Engineering ISSRE</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4132,7 +4078,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>url</t>
@@ -4163,7 +4108,6 @@
           <t>Wmsci 2006 the 10th World Multi Conference on Systemics Cybernetics and Informatics Jointly with the 12th International Conference on Information Systems Analysis and Synthesis Isas 2006 Proc</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>url</t>
@@ -4194,7 +4138,6 @@
           <t>Lecture Notes in Business Information Processing</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>url</t>
@@ -4220,14 +4163,11 @@
       <c r="C122" t="n">
         <v>2018</v>
       </c>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4248,7 +4188,6 @@
           <t>Proceedings of the International Conference on Software Engineering and Knowledge Engineering Seke</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>url</t>
@@ -4279,7 +4218,6 @@
           <t>Proceedings Annual Meeting of the Decision Sciences Institute</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>manifest_oa_found</t>
@@ -4310,7 +4248,11 @@
           <t>Proceedings Asia Pacific Software Engineering Conference APSEC</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F125" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4341,7 +4283,6 @@
           <t>Proceedings of the 27th Annual International Conference on Computer Science and Software Engineering Cascon 2017</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>url</t>
@@ -4407,7 +4348,11 @@
           <t>Proceedings of the 2008 IEEE Systems and Information Engineering Design Symposium Sieds 2008</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F128" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4438,7 +4383,6 @@
           <t>Icic Express Letters Part B Applications</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4469,7 +4413,6 @@
           <t>SN Computer Science</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4500,7 +4443,6 @@
           <t>Iet Conference Publications</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4531,7 +4473,6 @@
           <t>International Journal of Data Science and Analytics</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4562,7 +4503,6 @@
           <t>Communications in Computer and Information Science</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>url</t>
@@ -4593,7 +4533,6 @@
           <t>Icst 2010 3rd International Conference on Software Testing Verification and Validation</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4624,7 +4563,6 @@
           <t>17th International Conference on Software Engineering and Knowledge Engineering Seke 2005</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>url</t>
@@ -4655,7 +4593,6 @@
           <t>Empirical Software Engineering</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4686,7 +4623,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>url</t>
@@ -4717,7 +4653,11 @@
           <t>Esec Fse 2019 Proceedings of the 2019 27th ACM Joint Meeting European Software Engineering Conference and Symposium on the Foundations of Software Engineering</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4748,7 +4688,6 @@
           <t>Statistical Modelling</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>ft_oa_url</t>
@@ -4779,7 +4718,6 @@
           <t>International Journal of Managing Projects in Business</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4810,7 +4748,6 @@
           <t>Cibse 2014 Proceedings of the 17th Ibero American Conference Software Engineering</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>url</t>
@@ -4841,7 +4778,6 @@
           <t>Enase 2013 Proceedings of the 8th International Conference on Evaluation of Novel Approaches to Software Engineering</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>url</t>
@@ -4872,7 +4808,6 @@
           <t>Proceedings 2nd Asia Pacific Conference on Quality Software Apaqs 2001</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4903,7 +4838,6 @@
           <t>Ceur Workshop Proceedings</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>url</t>
@@ -4934,7 +4868,11 @@
           <t>Proceedings International Computer Software and Applications Conference</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="F145" t="inlineStr">
         <is>
           <t>doi</t>
@@ -4965,7 +4903,6 @@
           <t>Icsess 2011 Proceedings 2011 IEEE 2nd International Conference on Software Engineering and Service Science</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
           <t>doi</t>

</xml_diff>